<commit_message>
docs: BOM'da U4 için 74HCT125N alternatifi
74AHCT125N zor bulunuyor. Delikli kart için aynı bacak düzenli 74HCT125N
eklendi (giriş eşiği 2.0 V, 3.3 V veriyi okur); T'siz 74HC125'in neden
olmadığı not edildi. Excel yeniden üretildi.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014gmDZ9XSdHenPE7DWTzSSt
</commit_message>
<xml_diff>
--- a/docs/hardware/CC-BOM-01.xlsx
+++ b/docs/hardware/CC-BOM-01.xlsx
@@ -348,7 +348,7 @@
     <t xml:space="preserve">74AHCT1G125</t>
   </si>
   <si>
-    <t xml:space="preserve">SOT-23-5. Delikli kartta eşdeğer: 74AHCT125N (DIP-14)</t>
+    <t xml:space="preserve">SOT-23-5. Delikli kartta eşdeğer: 74HCT125N veya 74AHCT125N (DIP-14); 74HC125 olmaz</t>
   </si>
   <si>
     <t xml:space="preserve">3.3 V → 5 V seviye çevirici; OE → GND, VCC = +5V</t>
@@ -357,7 +357,7 @@
     <t xml:space="preserve">Önerilen</t>
   </si>
   <si>
-    <t xml:space="preserve">Seviye çevirici 74AHCT1G125 (veya 74AHCT125N)</t>
+    <t xml:space="preserve">Seviye çevirici 74AHCT1G125 (veya 74HCT125N / 74AHCT125N)</t>
   </si>
   <si>
     <t xml:space="preserve">R13</t>
@@ -936,7 +936,7 @@
     <t xml:space="preserve">1. WS2812B şerit katı (LS1, U4, R13, C8–C10, J4) şemada çizili değil; F2.4'te pins.h'e eklendi (GPIO27). Referanslar bu listede önerilmiştir.</t>
   </si>
   <si>
-    <t xml:space="preserve">2. D1 (SS34) ve U4 (74AHCT1G125) yüzey montajlıdır; kart delikli pertinaksa 1N5822 ve 74AHCT125N kullanılır.</t>
+    <t xml:space="preserve">2. D1 (SS34) ve U4 (74AHCT1G125) yüzey montajlıdır; kart delikli pertinaksa 1N5822 ve 74HCT125N (veya 74AHCT125N) kullanılır; T'siz 74HC125 3.3 V girişi güvenilir okumaz.</t>
   </si>
   <si>
     <t xml:space="preserve">3. Şema Sayfa 2 PE notundaki "U1 FG": IRM-10-5 Class II modüldür, FG pini yoktur.</t>
@@ -2265,7 +2265,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="n">
         <v>19</v>
       </c>
@@ -5727,7 +5727,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="36" t="s">
         <v>294</v>
       </c>

</xml_diff>